<commit_message>
chore: update overlap spreadsheets
</commit_message>
<xml_diff>
--- a/observations/capabilities/overlap.xlsx
+++ b/observations/capabilities/overlap.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="44">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="45">
   <si>
     <t>Capabilities</t>
   </si>
@@ -77,16 +77,19 @@
     <t>Ability to extend the web viewer with classic web extensions.</t>
   </si>
   <si>
+    <t>Inspect the contents of a web page.</t>
+  </si>
+  <si>
     <t>Open web pages in various web views/windows.</t>
   </si>
   <si>
     <t>Open web pages in various tabs or windows.</t>
   </si>
   <si>
-    <t>Inspect the contents of a web page. Though Peek does this better, regular browsers inspection tools are aimed at developers.</t>
-  </si>
-  <si>
-    <t>Inspect the contents of a web page.</t>
+    <t>Though Peek escapes the traditional browser window and provides a more tighter OS-level integration.</t>
+  </si>
+  <si>
+    <t>Darc is more similar to the browser in this regard, because it is based on IWAs, a web browser technology.</t>
   </si>
   <si>
     <t>Search the web without going to the search engine's web page first, keeping the web search tool close.</t>
@@ -151,7 +154,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="10">
+  <fonts count="11">
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
@@ -185,6 +188,12 @@
     <font>
       <b/>
       <color theme="4"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <name val="ui-sans-serif, system-ui, sans-serif, &quot;Apple Color Emoji&quot;, &quot;Segoe UI Emoji&quot;, Segoe UI Symbol, &quot;Noto Color Emoji&quot;"/>
+      <i/>
+      <color rgb="FF0c0c14"/>
     </font>
     <font>
       <b/>
@@ -221,7 +230,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -263,7 +272,7 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0">
@@ -273,6 +282,12 @@
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -480,7 +495,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D43"/>
+  <dimension ref="A1:D46"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="20.83" customWidth="1"/>
@@ -628,63 +643,61 @@
     <row r="18">
       <c r="A18" s="8"/>
       <c r="B18" s="14"/>
-      <c r="C18" t="s" s="14">
+      <c r="C18" t="s" s="15">
         <v>21</v>
       </c>
-      <c r="D18" t="s" s="14">
-        <v>22</v>
-      </c>
+      <c r="D18" s="15"/>
     </row>
     <row r="19">
       <c r="A19" s="8"/>
-      <c r="B19" s="14"/>
-      <c r="C19" t="s" s="14">
-        <v>23</v>
-      </c>
-      <c r="D19" t="s" s="14">
-        <v>24</v>
-      </c>
+      <c r="B19" s="8"/>
+      <c r="C19" s="8"/>
+      <c r="D19" s="8"/>
     </row>
     <row r="20">
       <c r="A20" s="8"/>
-      <c r="B20" s="8"/>
-      <c r="C20" s="8"/>
-      <c r="D20" s="8"/>
+      <c r="B20" s="14"/>
+      <c r="C20" t="s" s="8">
+        <v>22</v>
+      </c>
+      <c r="D20" t="s">
+        <v>23</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="8"/>
       <c r="B21" s="8"/>
-      <c r="C21" t="s" s="8">
+      <c r="C21" t="s" s="16">
+        <v>24</v>
+      </c>
+      <c r="D21" t="s" s="16">
         <v>25</v>
-      </c>
-      <c r="D21" t="s" s="8">
-        <v>26</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="8"/>
       <c r="B22" s="8"/>
-      <c r="C22" t="s" s="8">
-        <v>27</v>
-      </c>
-      <c r="D22" t="s" s="8">
-        <v>28</v>
-      </c>
+      <c r="C22" s="8"/>
+      <c r="D22" s="8"/>
     </row>
     <row r="23">
       <c r="A23" s="8"/>
       <c r="B23" s="8"/>
-      <c r="C23" s="8"/>
+      <c r="C23" t="s" s="8">
+        <v>26</v>
+      </c>
       <c r="D23" t="s" s="8">
-        <v>29</v>
+        <v>27</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="8"/>
       <c r="B24" s="8"/>
-      <c r="C24" s="8"/>
+      <c r="C24" t="s" s="8">
+        <v>28</v>
+      </c>
       <c r="D24" t="s" s="8">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="25">
@@ -692,61 +705,61 @@
       <c r="B25" s="8"/>
       <c r="C25" s="8"/>
       <c r="D25" t="s" s="8">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="8"/>
       <c r="B26" s="8"/>
       <c r="C26" s="8"/>
+      <c r="D26" t="s" s="8">
+        <v>31</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="8"/>
-      <c r="B27" s="12"/>
-      <c r="C27" s="12"/>
-    </row>
-    <row r="28" customHeight="1" ht="45">
+      <c r="B27" s="8"/>
+      <c r="C27" s="8"/>
+      <c r="D27" t="s" s="8">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="28">
       <c r="A28" s="8"/>
-      <c r="B28" s="12"/>
-      <c r="C28" t="s" s="12">
-        <v>32</v>
-      </c>
+      <c r="B28" s="8"/>
+      <c r="C28" s="8"/>
     </row>
     <row r="29">
       <c r="A29" s="8"/>
-      <c r="B29" s="15"/>
-      <c r="C29" t="s" s="15">
+      <c r="B29" s="12"/>
+      <c r="C29" s="12"/>
+    </row>
+    <row r="30" customHeight="1" ht="45">
+      <c r="A30" s="8"/>
+      <c r="B30" s="12"/>
+      <c r="C30" t="s" s="12">
         <v>33</v>
       </c>
-      <c r="D29" s="16"/>
-    </row>
-    <row r="30">
-      <c r="A30" s="8"/>
-      <c r="B30" s="8"/>
-      <c r="C30" s="8"/>
-      <c r="D30" s="8"/>
     </row>
     <row r="31">
       <c r="A31" s="8"/>
-      <c r="B31" s="8"/>
-      <c r="C31" t="s" s="8">
+      <c r="B31" s="17"/>
+      <c r="C31" t="s" s="17">
         <v>34</v>
       </c>
-      <c r="D31" s="8"/>
+      <c r="D31" s="18"/>
     </row>
     <row r="32">
       <c r="A32" s="8"/>
       <c r="B32" s="8"/>
-      <c r="C32" t="s" s="8">
-        <v>35</v>
-      </c>
+      <c r="C32" s="8"/>
       <c r="D32" s="8"/>
     </row>
     <row r="33">
       <c r="A33" s="8"/>
       <c r="B33" s="8"/>
       <c r="C33" t="s" s="8">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="D33" s="8"/>
     </row>
@@ -754,7 +767,7 @@
       <c r="A34" s="8"/>
       <c r="B34" s="8"/>
       <c r="C34" t="s" s="8">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D34" s="8"/>
     </row>
@@ -762,58 +775,75 @@
       <c r="A35" s="8"/>
       <c r="B35" s="8"/>
       <c r="C35" t="s" s="8">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="D35" s="8"/>
     </row>
     <row r="36">
+      <c r="A36" s="8"/>
       <c r="B36" s="8"/>
       <c r="C36" t="s" s="8">
+        <v>38</v>
+      </c>
+      <c r="D36" s="8"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="8"/>
+      <c r="B37" s="8"/>
+      <c r="C37" t="s" s="8">
         <v>39</v>
       </c>
-      <c r="D36" s="8"/>
+      <c r="D37" s="8"/>
     </row>
     <row r="38">
-      <c r="B38" s="12"/>
-      <c r="C38" s="12"/>
-    </row>
-    <row r="39" customHeight="1" ht="45">
-      <c r="B39" s="12"/>
-      <c r="C39" t="s" s="12">
+      <c r="B38" s="8"/>
+      <c r="C38" t="s" s="8">
         <v>40</v>
       </c>
+      <c r="D38" s="8"/>
     </row>
     <row r="40">
-      <c r="B40" s="17"/>
-      <c r="C40" t="s" s="17">
+      <c r="B40" s="12"/>
+      <c r="C40" s="12"/>
+    </row>
+    <row r="41" customHeight="1" ht="45">
+      <c r="B41" s="12"/>
+      <c r="C41" t="s" s="12">
         <v>41</v>
       </c>
-      <c r="D40" s="18"/>
     </row>
     <row r="42">
-      <c r="C42" t="s">
+      <c r="B42" s="19"/>
+      <c r="C42" t="s" s="19">
         <v>42</v>
       </c>
-    </row>
-    <row r="43">
-      <c r="C43" t="s">
+      <c r="D42" s="20"/>
+    </row>
+    <row r="44">
+      <c r="C44" t="s">
         <v>43</v>
       </c>
     </row>
+    <row r="45">
+      <c r="C45" t="s">
+        <v>44</v>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="12">
+  <mergeCells count="13">
     <mergeCell ref="C4:D4"/>
     <mergeCell ref="C5:D5"/>
     <mergeCell ref="C6:D6"/>
     <mergeCell ref="C7:D7"/>
     <mergeCell ref="C16:D16"/>
     <mergeCell ref="C17:D17"/>
-    <mergeCell ref="C28:D28"/>
-    <mergeCell ref="C29:D29"/>
-    <mergeCell ref="C31:D31"/>
-    <mergeCell ref="C39:D39"/>
-    <mergeCell ref="C40:D40"/>
-    <mergeCell ref="C42:D42"/>
+    <mergeCell ref="C18:D18"/>
+    <mergeCell ref="C32:D32"/>
+    <mergeCell ref="C33:D33"/>
+    <mergeCell ref="C35:D35"/>
+    <mergeCell ref="C43:D43"/>
+    <mergeCell ref="C44:D44"/>
+    <mergeCell ref="C46:D46"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>